<commit_message>
ci(dev): publish dev build from 53993e1579c054a480426ff1d55d8db64acdfb34 53993e1579c054a480426ff1d55d8db64acdfb34
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ph-core-doh-nhfr-code.xlsx
+++ b/dev/StructureDefinition-ph-core-doh-nhfr-code.xlsx
@@ -36,7 +36,7 @@
     <t>Name</t>
   </si>
   <si>
-    <t>PHCoreDohNhfrCode</t>
+    <t>PHCoreDOHNHFRCode</t>
   </si>
   <si>
     <t>Title</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-25T03:31:02+00:00</t>
+    <t>2026-03-25T03:34:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -422,7 +422,7 @@
     <t>There are many sets  of identifiers.  To perform matching of two identifiers, we need to know what set we're dealing with. The system identifies a particular set of unique identifiers.</t>
   </si>
   <si>
-    <t>http://doh.gov.ph/fhir/ph-core/NamingSystem/doh-nhfr-code-ns</t>
+    <t>http://doh.gov.ph/fhir/Identifier/doh-nhfr-code</t>
   </si>
   <si>
     <t>http://www.acme.com/identifiers/patient</t>

</xml_diff>